<commit_message>
add carrier, bios, sym, readme
</commit_message>
<xml_diff>
--- a/Electricals/Pinouts/LattePanda_Mu_Edge_Connector_Pinout.xlsx
+++ b/Electricals/Pinouts/LattePanda_Mu_Edge_Connector_Pinout.xlsx
@@ -1,10 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitHub\LattePanda-Mu\Electricals\Pinouts\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="27945" windowHeight="12375" activeTab="1"/>
+    <workbookView windowWidth="27945" windowHeight="12375"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="4" r:id="rId1"/>
@@ -33,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1442" uniqueCount="355">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1442" uniqueCount="357">
   <si>
     <r>
       <rPr>
@@ -627,6 +632,9 @@
     <t>DDIB_AUX_N</t>
   </si>
   <si>
+    <t>0.6V</t>
+  </si>
+  <si>
     <t>DDIB DP Auxiliary Channel</t>
   </si>
   <si>
@@ -634,6 +642,9 @@
   </si>
   <si>
     <t>DDIB_TX3_N</t>
+  </si>
+  <si>
+    <t>1.2V</t>
   </si>
   <si>
     <t>DDIB DP Lane 3 / HDMI TMDS Clock</t>
@@ -4683,10 +4694,10 @@
         <v>68</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>17</v>
+        <v>168</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F98" s="2" t="s">
         <v>19</v>
@@ -4697,16 +4708,16 @@
         <v>193</v>
       </c>
       <c r="B99" s="2" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C99" s="3" t="s">
         <v>68</v>
       </c>
       <c r="D99" s="2" t="s">
-        <v>17</v>
+        <v>168</v>
       </c>
       <c r="E99" s="2" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F99" s="2" t="s">
         <v>19</v>
@@ -4737,16 +4748,16 @@
         <v>197</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C101" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="F101" s="2" t="s">
         <v>40</v>
@@ -4760,16 +4771,16 @@
         <v>199</v>
       </c>
       <c r="B102" s="2" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="C102" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D102" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E102" s="2" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="F102" s="2" t="s">
         <v>40</v>
@@ -4803,16 +4814,16 @@
         <v>203</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C104" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F104" s="2" t="s">
         <v>40</v>
@@ -4826,16 +4837,16 @@
         <v>205</v>
       </c>
       <c r="B105" s="2" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C105" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D105" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E105" s="2" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F105" s="2" t="s">
         <v>40</v>
@@ -4869,16 +4880,16 @@
         <v>209</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C107" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F107" s="2" t="s">
         <v>40</v>
@@ -4892,16 +4903,16 @@
         <v>211</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C108" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D108" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E108" s="2" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F108" s="2" t="s">
         <v>40</v>
@@ -4935,16 +4946,16 @@
         <v>215</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C110" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E110" s="2" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F110" s="2" t="s">
         <v>40</v>
@@ -4958,16 +4969,16 @@
         <v>217</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C111" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D111" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E111" s="2" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="F111" s="2" t="s">
         <v>40</v>
@@ -5001,16 +5012,16 @@
         <v>221</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C113" s="3" t="s">
         <v>68</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>17</v>
+        <v>168</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="F113" s="2" t="s">
         <v>19</v>
@@ -5021,16 +5032,16 @@
         <v>223</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C114" s="3" t="s">
         <v>68</v>
       </c>
       <c r="D114" s="2" t="s">
-        <v>17</v>
+        <v>168</v>
       </c>
       <c r="E114" s="2" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="F114" s="2" t="s">
         <v>19</v>
@@ -5061,16 +5072,16 @@
         <v>227</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="C116" s="3" t="s">
         <v>68</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F116" s="2" t="s">
         <v>40</v>
@@ -5084,16 +5095,16 @@
         <v>229</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C117" s="3" t="s">
         <v>68</v>
       </c>
       <c r="D117" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E117" s="2" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="F117" s="2" t="s">
         <v>40</v>
@@ -5127,16 +5138,16 @@
         <v>233</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="C119" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E119" s="2" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F119" s="2" t="s">
         <v>40</v>
@@ -5150,16 +5161,16 @@
         <v>235</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C120" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D120" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E120" s="2" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F120" s="2" t="s">
         <v>40</v>
@@ -5193,16 +5204,16 @@
         <v>239</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C122" s="3" t="s">
         <v>68</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E122" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="F122" s="2" t="s">
         <v>40</v>
@@ -5216,16 +5227,16 @@
         <v>241</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C123" s="3" t="s">
         <v>68</v>
       </c>
       <c r="D123" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E123" s="2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="F123" s="2" t="s">
         <v>40</v>
@@ -5259,16 +5270,16 @@
         <v>245</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C125" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E125" s="2" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F125" s="2" t="s">
         <v>40</v>
@@ -5282,16 +5293,16 @@
         <v>247</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C126" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D126" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E126" s="2" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F126" s="2" t="s">
         <v>40</v>
@@ -5325,16 +5336,16 @@
         <v>251</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C128" s="3" t="s">
         <v>33</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E128" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F128" s="2" t="s">
         <v>36</v>
@@ -5345,16 +5356,16 @@
         <v>253</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C129" s="3" t="s">
         <v>33</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E129" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F129" s="2" t="s">
         <v>36</v>
@@ -5365,16 +5376,16 @@
         <v>255</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C130" s="3" t="s">
         <v>33</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E130" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F130" s="2" t="s">
         <v>36</v>
@@ -5385,16 +5396,16 @@
         <v>257</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C131" s="3" t="s">
         <v>33</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E131" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F131" s="2" t="s">
         <v>36</v>
@@ -5405,16 +5416,16 @@
         <v>259</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C132" s="3" t="s">
         <v>33</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E132" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F132" s="2" t="s">
         <v>36</v>
@@ -5475,7 +5486,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>24</v>
@@ -5484,13 +5495,13 @@
         <v>17</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="3" spans="1:7">
@@ -5498,16 +5509,16 @@
         <v>4</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="F3" s="2" t="s">
         <v>19</v>
@@ -5518,7 +5529,7 @@
         <v>6</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>24</v>
@@ -5527,13 +5538,13 @@
         <v>17</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="F4" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -5541,16 +5552,16 @@
         <v>8</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C5" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F5" s="2" t="s">
         <v>19</v>
@@ -5561,7 +5572,7 @@
         <v>10</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>24</v>
@@ -5570,7 +5581,7 @@
         <v>17</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="F6" s="2" t="s">
         <v>19</v>
@@ -5581,7 +5592,7 @@
         <v>12</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>16</v>
@@ -5590,7 +5601,7 @@
         <v>17</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="F7" s="2" t="s">
         <v>19</v>
@@ -5621,7 +5632,7 @@
         <v>16</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>16</v>
@@ -5630,7 +5641,7 @@
         <v>38</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F9" s="2" t="s">
         <v>40</v>
@@ -5644,7 +5655,7 @@
         <v>18</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>16</v>
@@ -5653,7 +5664,7 @@
         <v>38</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>40</v>
@@ -5687,7 +5698,7 @@
         <v>22</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C12" s="3" t="s">
         <v>16</v>
@@ -5696,7 +5707,7 @@
         <v>38</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="F12" s="2" t="s">
         <v>40</v>
@@ -5710,7 +5721,7 @@
         <v>24</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>16</v>
@@ -5719,7 +5730,7 @@
         <v>38</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="F13" s="2" t="s">
         <v>40</v>
@@ -5753,7 +5764,7 @@
         <v>28</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="C15" s="3" t="s">
         <v>16</v>
@@ -5762,7 +5773,7 @@
         <v>38</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="F15" s="2" t="s">
         <v>40</v>
@@ -5776,7 +5787,7 @@
         <v>30</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C16" s="3" t="s">
         <v>16</v>
@@ -5785,7 +5796,7 @@
         <v>38</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>40</v>
@@ -5819,7 +5830,7 @@
         <v>34</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C18" s="3" t="s">
         <v>16</v>
@@ -5828,7 +5839,7 @@
         <v>38</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F18" s="2" t="s">
         <v>40</v>
@@ -5842,7 +5853,7 @@
         <v>36</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C19" s="3" t="s">
         <v>16</v>
@@ -5851,7 +5862,7 @@
         <v>38</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>40</v>
@@ -5885,7 +5896,7 @@
         <v>40</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C21" s="3" t="s">
         <v>16</v>
@@ -5894,7 +5905,7 @@
         <v>38</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>40</v>
@@ -5908,7 +5919,7 @@
         <v>42</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="C22" s="3" t="s">
         <v>16</v>
@@ -5917,7 +5928,7 @@
         <v>38</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="F22" s="2" t="s">
         <v>40</v>
@@ -5951,7 +5962,7 @@
         <v>46</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="C24" s="3" t="s">
         <v>16</v>
@@ -5960,7 +5971,7 @@
         <v>38</v>
       </c>
       <c r="E24" s="2" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="F24" s="2" t="s">
         <v>40</v>
@@ -5974,7 +5985,7 @@
         <v>48</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>16</v>
@@ -5983,7 +5994,7 @@
         <v>38</v>
       </c>
       <c r="E25" s="2" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="F25" s="2" t="s">
         <v>40</v>
@@ -6017,7 +6028,7 @@
         <v>52</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="C27" s="3" t="s">
         <v>16</v>
@@ -6026,7 +6037,7 @@
         <v>38</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="F27" s="2" t="s">
         <v>40</v>
@@ -6040,7 +6051,7 @@
         <v>54</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C28" s="3" t="s">
         <v>16</v>
@@ -6049,7 +6060,7 @@
         <v>38</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="F28" s="2" t="s">
         <v>40</v>
@@ -6083,7 +6094,7 @@
         <v>58</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="C30" s="3" t="s">
         <v>16</v>
@@ -6092,7 +6103,7 @@
         <v>38</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="F30" s="2" t="s">
         <v>40</v>
@@ -6106,7 +6117,7 @@
         <v>60</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="C31" s="3" t="s">
         <v>16</v>
@@ -6115,7 +6126,7 @@
         <v>38</v>
       </c>
       <c r="E31" s="2" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>40</v>
@@ -6149,7 +6160,7 @@
         <v>64</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="C33" s="3" t="s">
         <v>16</v>
@@ -6158,7 +6169,7 @@
         <v>38</v>
       </c>
       <c r="E33" s="2" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="F33" s="2" t="s">
         <v>40</v>
@@ -6172,7 +6183,7 @@
         <v>66</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>16</v>
@@ -6181,7 +6192,7 @@
         <v>38</v>
       </c>
       <c r="E34" s="2" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="F34" s="2" t="s">
         <v>40</v>
@@ -6215,7 +6226,7 @@
         <v>70</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>68</v>
@@ -6224,7 +6235,7 @@
         <v>69</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="F36" s="2" t="s">
         <v>40</v>
@@ -6235,7 +6246,7 @@
         <v>72</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>68</v>
@@ -6244,7 +6255,7 @@
         <v>69</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="F37" s="2" t="s">
         <v>40</v>
@@ -6275,7 +6286,7 @@
         <v>76</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="C39" s="3" t="s">
         <v>68</v>
@@ -6284,7 +6295,7 @@
         <v>69</v>
       </c>
       <c r="E39" s="2" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="F39" s="2" t="s">
         <v>40</v>
@@ -6295,7 +6306,7 @@
         <v>78</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="C40" s="3" t="s">
         <v>68</v>
@@ -6304,7 +6315,7 @@
         <v>69</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="F40" s="2" t="s">
         <v>40</v>
@@ -6335,7 +6346,7 @@
         <v>82</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C42" s="3" t="s">
         <v>68</v>
@@ -6344,7 +6355,7 @@
         <v>69</v>
       </c>
       <c r="E42" s="2" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="F42" s="2" t="s">
         <v>40</v>
@@ -6355,7 +6366,7 @@
         <v>84</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>68</v>
@@ -6364,7 +6375,7 @@
         <v>69</v>
       </c>
       <c r="E43" s="2" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="F43" s="2" t="s">
         <v>40</v>
@@ -6395,7 +6406,7 @@
         <v>88</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C45" s="3" t="s">
         <v>24</v>
@@ -6404,7 +6415,7 @@
         <v>38</v>
       </c>
       <c r="E45" s="2" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="F45" s="2" t="s">
         <v>40</v>
@@ -6418,7 +6429,7 @@
         <v>90</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="C46" s="3" t="s">
         <v>24</v>
@@ -6427,7 +6438,7 @@
         <v>38</v>
       </c>
       <c r="E46" s="2" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="F46" s="2" t="s">
         <v>40</v>
@@ -6461,7 +6472,7 @@
         <v>94</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="C48" s="3" t="s">
         <v>24</v>
@@ -6470,7 +6481,7 @@
         <v>38</v>
       </c>
       <c r="E48" s="2" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="F48" s="2" t="s">
         <v>40</v>
@@ -6484,7 +6495,7 @@
         <v>96</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C49" s="3" t="s">
         <v>24</v>
@@ -6493,7 +6504,7 @@
         <v>38</v>
       </c>
       <c r="E49" s="2" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="F49" s="2" t="s">
         <v>40</v>
@@ -6527,7 +6538,7 @@
         <v>100</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="C51" s="3" t="s">
         <v>16</v>
@@ -6536,7 +6547,7 @@
         <v>69</v>
       </c>
       <c r="E51" s="2" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="F51" s="2" t="s">
         <v>19</v>
@@ -6550,7 +6561,7 @@
         <v>102</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C52" s="3" t="s">
         <v>16</v>
@@ -6559,7 +6570,7 @@
         <v>69</v>
       </c>
       <c r="E52" s="2" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="F52" s="2" t="s">
         <v>19</v>
@@ -6573,7 +6584,7 @@
         <v>104</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="C53" s="3" t="s">
         <v>16</v>
@@ -6582,7 +6593,7 @@
         <v>69</v>
       </c>
       <c r="E53" s="2" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="F53" s="2" t="s">
         <v>19</v>
@@ -6596,7 +6607,7 @@
         <v>106</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="C54" s="3" t="s">
         <v>24</v>
@@ -6605,7 +6616,7 @@
         <v>69</v>
       </c>
       <c r="E54" s="2" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="F54" s="2" t="s">
         <v>19</v>
@@ -6619,7 +6630,7 @@
         <v>108</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="C55" s="3" t="s">
         <v>68</v>
@@ -6628,7 +6639,7 @@
         <v>69</v>
       </c>
       <c r="E55" s="2" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="F55" s="2" t="s">
         <v>19</v>
@@ -6662,7 +6673,7 @@
         <v>112</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="C57" s="3" t="s">
         <v>68</v>
@@ -6671,7 +6682,7 @@
         <v>69</v>
       </c>
       <c r="E57" s="2" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="F57" s="2" t="s">
         <v>40</v>
@@ -6682,7 +6693,7 @@
         <v>114</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C58" s="3" t="s">
         <v>68</v>
@@ -6691,7 +6702,7 @@
         <v>69</v>
       </c>
       <c r="E58" s="2" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="F58" s="2" t="s">
         <v>40</v>
@@ -6722,7 +6733,7 @@
         <v>118</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="C60" s="3" t="s">
         <v>68</v>
@@ -6742,7 +6753,7 @@
         <v>120</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="C61" s="3" t="s">
         <v>68</v>
@@ -6762,7 +6773,7 @@
         <v>122</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="C62" s="3" t="s">
         <v>68</v>
@@ -6782,7 +6793,7 @@
         <v>124</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C63" s="3" t="s">
         <v>68</v>
@@ -6802,7 +6813,7 @@
         <v>126</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="C64" s="3" t="s">
         <v>68</v>
@@ -6822,7 +6833,7 @@
         <v>128</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="C65" s="3" t="s">
         <v>68</v>
@@ -6845,7 +6856,7 @@
         <v>130</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C66" s="3" t="s">
         <v>68</v>
@@ -6860,7 +6871,7 @@
         <v>19</v>
       </c>
       <c r="G66" s="2" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
     </row>
     <row r="67" spans="1:7">
@@ -6868,7 +6879,7 @@
         <v>132</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C67" s="3" t="s">
         <v>68</v>
@@ -6883,7 +6894,7 @@
         <v>19</v>
       </c>
       <c r="G67" s="2" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="68" spans="1:7">
@@ -6891,7 +6902,7 @@
         <v>134</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="C68" s="3" t="s">
         <v>68</v>
@@ -6934,7 +6945,7 @@
         <v>138</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C70" s="3" t="s">
         <v>68</v>
@@ -6943,7 +6954,7 @@
         <v>17</v>
       </c>
       <c r="E70" s="2" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="F70" s="2" t="s">
         <v>19</v>
@@ -6957,7 +6968,7 @@
         <v>140</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C71" s="3" t="s">
         <v>68</v>
@@ -6966,7 +6977,7 @@
         <v>17</v>
       </c>
       <c r="E71" s="2" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="F71" s="2" t="s">
         <v>19</v>
@@ -6980,7 +6991,7 @@
         <v>142</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C72" s="3" t="s">
         <v>24</v>
@@ -6989,7 +7000,7 @@
         <v>69</v>
       </c>
       <c r="E72" s="2" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="F72" s="2" t="s">
         <v>19</v>
@@ -7003,7 +7014,7 @@
         <v>144</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="C73" s="3" t="s">
         <v>68</v>
@@ -7012,7 +7023,7 @@
         <v>69</v>
       </c>
       <c r="E73" s="2" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="F73" s="2" t="s">
         <v>19</v>
@@ -7037,7 +7048,7 @@
         <v>146</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="C75" s="3" t="s">
         <v>24</v>
@@ -7046,7 +7057,7 @@
         <v>69</v>
       </c>
       <c r="E75" s="2" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="F75" s="2" t="s">
         <v>19</v>
@@ -7060,7 +7071,7 @@
         <v>148</v>
       </c>
       <c r="B76" s="2" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="C76" s="3" t="s">
         <v>68</v>
@@ -7069,7 +7080,7 @@
         <v>69</v>
       </c>
       <c r="E76" s="2" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="F76" s="2" t="s">
         <v>19</v>
@@ -7083,7 +7094,7 @@
         <v>150</v>
       </c>
       <c r="B77" s="2" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="C77" s="3" t="s">
         <v>24</v>
@@ -7092,7 +7103,7 @@
         <v>69</v>
       </c>
       <c r="E77" s="2" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="F77" s="2" t="s">
         <v>19</v>
@@ -7106,7 +7117,7 @@
         <v>152</v>
       </c>
       <c r="B78" s="2" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="C78" s="3" t="s">
         <v>68</v>
@@ -7115,7 +7126,7 @@
         <v>69</v>
       </c>
       <c r="E78" s="2" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="F78" s="2" t="s">
         <v>19</v>
@@ -7129,7 +7140,7 @@
         <v>154</v>
       </c>
       <c r="B79" s="2" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C79" s="3" t="s">
         <v>24</v>
@@ -7138,7 +7149,7 @@
         <v>69</v>
       </c>
       <c r="E79" s="2" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="F79" s="2" t="s">
         <v>19</v>
@@ -7152,7 +7163,7 @@
         <v>156</v>
       </c>
       <c r="B80" s="2" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="C80" s="3" t="s">
         <v>68</v>
@@ -7161,7 +7172,7 @@
         <v>69</v>
       </c>
       <c r="E80" s="2" t="s">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="F80" s="2" t="s">
         <v>19</v>
@@ -7195,16 +7206,16 @@
         <v>160</v>
       </c>
       <c r="B82" s="2" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="C82" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E82" s="2" t="s">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="F82" s="2" t="s">
         <v>19</v>
@@ -7215,16 +7226,16 @@
         <v>162</v>
       </c>
       <c r="B83" s="2" t="s">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="C83" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D83" s="2" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E83" s="2" t="s">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="F83" s="2" t="s">
         <v>19</v>
@@ -7235,16 +7246,16 @@
         <v>164</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="C84" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D84" s="2" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E84" s="2" t="s">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="F84" s="2" t="s">
         <v>19</v>
@@ -7255,16 +7266,16 @@
         <v>166</v>
       </c>
       <c r="B85" s="2" t="s">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="C85" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D85" s="2" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E85" s="2" t="s">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="F85" s="2" t="s">
         <v>19</v>
@@ -7275,16 +7286,16 @@
         <v>168</v>
       </c>
       <c r="B86" s="2" t="s">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="C86" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D86" s="2" t="s">
-        <v>301</v>
+        <v>303</v>
       </c>
       <c r="E86" s="2" t="s">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="F86" s="2" t="s">
         <v>19</v>
@@ -7315,7 +7326,7 @@
         <v>172</v>
       </c>
       <c r="B88" s="2" t="s">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="C88" s="3" t="s">
         <v>24</v>
@@ -7324,7 +7335,7 @@
         <v>69</v>
       </c>
       <c r="E88" s="2" t="s">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="F88" s="2" t="s">
         <v>19</v>
@@ -7335,7 +7346,7 @@
         <v>174</v>
       </c>
       <c r="B89" s="2" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="C89" s="3" t="s">
         <v>24</v>
@@ -7344,7 +7355,7 @@
         <v>69</v>
       </c>
       <c r="E89" s="2" t="s">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="F89" s="2" t="s">
         <v>19</v>
@@ -7355,7 +7366,7 @@
         <v>176</v>
       </c>
       <c r="B90" s="2" t="s">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="C90" s="3" t="s">
         <v>24</v>
@@ -7364,7 +7375,7 @@
         <v>69</v>
       </c>
       <c r="E90" s="2" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="F90" s="2" t="s">
         <v>19</v>
@@ -7375,7 +7386,7 @@
         <v>178</v>
       </c>
       <c r="B91" s="2" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="C91" s="3" t="s">
         <v>24</v>
@@ -7384,7 +7395,7 @@
         <v>69</v>
       </c>
       <c r="E91" s="2" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="F91" s="2" t="s">
         <v>19</v>
@@ -7395,7 +7406,7 @@
         <v>180</v>
       </c>
       <c r="B92" s="2" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="C92" s="3" t="s">
         <v>16</v>
@@ -7404,7 +7415,7 @@
         <v>69</v>
       </c>
       <c r="E92" s="2" t="s">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="F92" s="2" t="s">
         <v>19</v>
@@ -7435,16 +7446,16 @@
         <v>184</v>
       </c>
       <c r="B94" s="2" t="s">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="C94" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D94" s="2" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E94" s="2" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="F94" s="2" t="s">
         <v>40</v>
@@ -7455,16 +7466,16 @@
         <v>186</v>
       </c>
       <c r="B95" s="2" t="s">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="C95" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D95" s="2" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E95" s="2" t="s">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="F95" s="2" t="s">
         <v>40</v>
@@ -7495,16 +7506,16 @@
         <v>190</v>
       </c>
       <c r="B97" s="2" t="s">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="C97" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="F97" s="2" t="s">
         <v>40</v>
@@ -7515,16 +7526,16 @@
         <v>192</v>
       </c>
       <c r="B98" s="2" t="s">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="C98" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D98" s="2" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E98" s="2" t="s">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="F98" s="2" t="s">
         <v>40</v>
@@ -7555,16 +7566,16 @@
         <v>196</v>
       </c>
       <c r="B100" s="2" t="s">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="C100" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D100" s="2" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E100" s="2" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="F100" s="2" t="s">
         <v>40</v>
@@ -7575,16 +7586,16 @@
         <v>198</v>
       </c>
       <c r="B101" s="2" t="s">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C101" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D101" s="2" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E101" s="2" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="F101" s="2" t="s">
         <v>40</v>
@@ -7615,16 +7626,16 @@
         <v>202</v>
       </c>
       <c r="B103" s="2" t="s">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="C103" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D103" s="2" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E103" s="2" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="F103" s="2" t="s">
         <v>40</v>
@@ -7635,16 +7646,16 @@
         <v>204</v>
       </c>
       <c r="B104" s="2" t="s">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="C104" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D104" s="2" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E104" s="2" t="s">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="F104" s="2" t="s">
         <v>40</v>
@@ -7675,16 +7686,16 @@
         <v>208</v>
       </c>
       <c r="B106" s="2" t="s">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="C106" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D106" s="2" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E106" s="2" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="F106" s="2" t="s">
         <v>40</v>
@@ -7695,16 +7706,16 @@
         <v>210</v>
       </c>
       <c r="B107" s="2" t="s">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="C107" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D107" s="2" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E107" s="2" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="F107" s="2" t="s">
         <v>40</v>
@@ -7735,16 +7746,16 @@
         <v>214</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="C109" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D109" s="2" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E109" s="2" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="F109" s="2" t="s">
         <v>40</v>
@@ -7755,16 +7766,16 @@
         <v>216</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="C110" s="3" t="s">
         <v>16</v>
       </c>
       <c r="D110" s="2" t="s">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="E110" s="2" t="s">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="F110" s="2" t="s">
         <v>40</v>
@@ -7795,16 +7806,16 @@
         <v>220</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="C112" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D112" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E112" s="2" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="F112" s="2" t="s">
         <v>40</v>
@@ -7818,16 +7829,16 @@
         <v>222</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="C113" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D113" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E113" s="2" t="s">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="F113" s="2" t="s">
         <v>40</v>
@@ -7861,16 +7872,16 @@
         <v>226</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="C115" s="3" t="s">
         <v>68</v>
       </c>
       <c r="D115" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E115" s="2" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="F115" s="2" t="s">
         <v>40</v>
@@ -7884,16 +7895,16 @@
         <v>228</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="C116" s="3" t="s">
         <v>68</v>
       </c>
       <c r="D116" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E116" s="2" t="s">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="F116" s="2" t="s">
         <v>40</v>
@@ -7927,16 +7938,16 @@
         <v>232</v>
       </c>
       <c r="B118" s="2" t="s">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C118" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D118" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E118" s="2" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="F118" s="2" t="s">
         <v>40</v>
@@ -7950,16 +7961,16 @@
         <v>234</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="C119" s="3" t="s">
         <v>24</v>
       </c>
       <c r="D119" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E119" s="2" t="s">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="F119" s="2" t="s">
         <v>40</v>
@@ -7993,16 +8004,16 @@
         <v>238</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="C121" s="3" t="s">
         <v>68</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E121" s="2" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="F121" s="2" t="s">
         <v>40</v>
@@ -8016,16 +8027,16 @@
         <v>240</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="C122" s="3" t="s">
         <v>68</v>
       </c>
       <c r="D122" s="2" t="s">
-        <v>17</v>
+        <v>172</v>
       </c>
       <c r="E122" s="2" t="s">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="F122" s="2" t="s">
         <v>40</v>
@@ -8059,16 +8070,16 @@
         <v>244</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="C124" s="3" t="s">
         <v>68</v>
       </c>
       <c r="D124" s="2" t="s">
-        <v>17</v>
+        <v>168</v>
       </c>
       <c r="E124" s="2" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="F124" s="2" t="s">
         <v>19</v>
@@ -8079,16 +8090,16 @@
         <v>246</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C125" s="3" t="s">
         <v>68</v>
       </c>
       <c r="D125" s="2" t="s">
-        <v>17</v>
+        <v>168</v>
       </c>
       <c r="E125" s="2" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="F125" s="2" t="s">
         <v>19</v>
@@ -8119,16 +8130,16 @@
         <v>250</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C127" s="3" t="s">
         <v>33</v>
       </c>
       <c r="D127" s="2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E127" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F127" s="2" t="s">
         <v>36</v>
@@ -8139,16 +8150,16 @@
         <v>252</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C128" s="3" t="s">
         <v>33</v>
       </c>
       <c r="D128" s="2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E128" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F128" s="2" t="s">
         <v>36</v>
@@ -8159,16 +8170,16 @@
         <v>254</v>
       </c>
       <c r="B129" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C129" s="3" t="s">
         <v>33</v>
       </c>
       <c r="D129" s="2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E129" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F129" s="2" t="s">
         <v>36</v>
@@ -8179,16 +8190,16 @@
         <v>256</v>
       </c>
       <c r="B130" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C130" s="3" t="s">
         <v>33</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E130" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F130" s="2" t="s">
         <v>36</v>
@@ -8199,16 +8210,16 @@
         <v>258</v>
       </c>
       <c r="B131" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C131" s="3" t="s">
         <v>33</v>
       </c>
       <c r="D131" s="2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E131" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F131" s="2" t="s">
         <v>36</v>
@@ -8219,16 +8230,16 @@
         <v>260</v>
       </c>
       <c r="B132" s="2" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C132" s="3" t="s">
         <v>33</v>
       </c>
       <c r="D132" s="2" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="E132" s="2" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="F132" s="2" t="s">
         <v>36</v>

</xml_diff>